<commit_message>
Add invoice reference per HS code to the summary sheet
New "Faktura / Invoice" column on Souhrn-HS lists which invoice(s) each HS
code draws on and how much value comes from each - needed to reference the
right invoice per item on the JSD. All three main codes span both invoices;
only the unresolved type wheel is single-invoice.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjrBV2HCzRFVHdsJfaktnd
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MOREK_CZ_CZ26008741.xlsx
+++ b/output/HS_Code_Summary_MOREK_CZ_CZ26008741.xlsx
@@ -621,20 +621,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -789,45 +790,50 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
+          <t>Faktura / Invoice (hodnota USD)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
           <t>Popis zboží (CZ)</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Description (EN)</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Čistá hm. / Net (kg)</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Hrubá hm. / Gross (kg)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Množství / Qty</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>MJ / Unit</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Celní hodnota / Customs value (USD)</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -846,41 +852,47 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
+          <t>CI-26051504: 22 100,66
+CI-26051902: 376,69</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
           <t>Smršťovací trubice silnostěnná a středněstěnná — Izolace, ochrana a vnější těsnění pro kabely níz. a stř. napětí</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Heat-shrink tubing, heavywall and mediumwall (with and without adhesive liner) — insulation, protection and outer sealing for LV/MV cables</t>
         </is>
       </c>
-      <c r="E16" s="7">
+      <c r="F16" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"HW")+SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-A")+SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-U")</f>
         <v>2978.58</v>
       </c>
-      <c r="F16" s="7">
+      <c r="G16" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"HW")+SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-A")+SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-U")</f>
         <v>3452.37</v>
       </c>
-      <c r="G16" s="8">
+      <c r="H16" s="8">
         <f>SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"HW")+SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-A")+SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-U")</f>
         <v>28935.0</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>ks / pcs</t>
         </is>
       </c>
-      <c r="I16" s="7">
+      <c r="J16" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"HW")+SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-A")+SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"MW-U")</f>
         <v>22477.35</v>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Ne / No</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>Ne / No — žádné opatření nezjištěno</t>
         </is>
@@ -899,41 +911,47 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
+          <t>CI-26051504: 6 347,52
+CI-26051902: 17 612,08</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
           <t>Spojovací set — Izolace a ochrana pro kabely nízkého napětí</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>MSTS cable jointing/termination kits — insulation and protection for LV cables</t>
         </is>
       </c>
-      <c r="E17" s="7">
+      <c r="F17" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"KIT")</f>
         <v>4488.82</v>
       </c>
-      <c r="F17" s="7">
+      <c r="G17" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"KIT")</f>
         <v>5415.63</v>
       </c>
-      <c r="G17" s="8">
+      <c r="H17" s="8">
         <f>SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"KIT")</f>
         <v>9530.0</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>sada / kit</t>
         </is>
       </c>
-      <c r="I17" s="7">
+      <c r="J17" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"KIT")</f>
         <v>23959.6</v>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Ne / No</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>Ne / No — žádné opatření nezjištěno</t>
         </is>
@@ -952,41 +970,47 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
+          <t>CI-26051504: 14 385,43
+CI-26051902: 6 120,94</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
           <t>Smršťovací bužírka tenkostěnná — Izolace a ochrana pro kabely nízkého napětí</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Thinwall heat-shrink sleeving 2:1 — insulation and protection for LV cables</t>
         </is>
       </c>
-      <c r="E18" s="7">
+      <c r="F18" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"TW")</f>
         <v>2175.6</v>
       </c>
-      <c r="F18" s="7">
+      <c r="G18" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"TW")</f>
         <v>2562.0</v>
       </c>
-      <c r="G18" s="8">
+      <c r="H18" s="8">
         <f>SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"TW")</f>
         <v>96740.0</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>ks / m</t>
         </is>
       </c>
-      <c r="I18" s="7">
+      <c r="J18" s="7">
         <f>SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"TW")</f>
         <v>20506.37</v>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Ne / No</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>Ne / No — žádné opatření nezjištěno</t>
         </is>
@@ -1005,41 +1029,46 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
+          <t>CI-26051504: 120,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
           <t>Tiskové (značkovací) kolečko — není v e-mailu ani v balicím listu, nutno doplnit (viz Poznámky, bod 6)</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Type wheel (printing/marking wheel) — absent from both the forwarder's code list and the packing list; needs identification</t>
         </is>
       </c>
-      <c r="E19" s="10">
+      <c r="F19" s="10">
         <f>SUMIFS('Rozpad-dle-produktu'!$I$10:$I$18,'Rozpad-dle-produktu'!$C$10:$C$18,"OTH")</f>
         <v>0.0</v>
       </c>
-      <c r="F19" s="10">
+      <c r="G19" s="10">
         <f>SUMIFS('Rozpad-dle-produktu'!$J$10:$J$18,'Rozpad-dle-produktu'!$C$10:$C$18,"OTH")</f>
         <v>0.0</v>
       </c>
-      <c r="G19" s="11">
+      <c r="H19" s="11">
         <f>SUMIFS('Rozpad-dle-produktu'!$G$10:$G$18,'Rozpad-dle-produktu'!$C$10:$C$18,"OTH")</f>
         <v>3.0</v>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="I19" s="9" t="inlineStr">
         <is>
           <t>ks / pcs</t>
         </is>
       </c>
-      <c r="I19" s="10">
+      <c r="J19" s="10">
         <f>SUMIFS('Rozpad-dle-produktu'!$K$10:$K$18,'Rozpad-dle-produktu'!$C$10:$C$18,"OTH")</f>
         <v>120.0</v>
       </c>
-      <c r="J19" s="9" t="inlineStr">
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>Ne / No</t>
         </is>
       </c>
-      <c r="K19" s="9" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>Ne / No</t>
         </is>
@@ -1049,30 +1078,31 @@
       <c r="A20" s="12" t="n"/>
       <c r="B20" s="12" t="n"/>
       <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>CELKEM / TOTAL</t>
         </is>
-      </c>
-      <c r="E20" s="13">
-        <f>SUM(E16:E19)</f>
-        <v>9643.0</v>
       </c>
       <c r="F20" s="13">
         <f>SUM(F16:F19)</f>
+        <v>9643.0</v>
+      </c>
+      <c r="G20" s="13">
+        <f>SUM(G16:G19)</f>
         <v>11430.0</v>
       </c>
-      <c r="G20" s="14">
-        <f>SUM(G16:G19)</f>
+      <c r="H20" s="14">
+        <f>SUM(H16:H19)</f>
         <v>135208.0</v>
       </c>
-      <c r="H20" s="12" t="n"/>
-      <c r="I20" s="13">
-        <f>SUM(I16:I19)</f>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="13">
+        <f>SUM(J16:J19)</f>
         <v>67063.32</v>
       </c>
-      <c r="J20" s="12" t="n"/>
       <c r="K20" s="12" t="n"/>
+      <c r="L20" s="12" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -1087,15 +1117,15 @@
           <t>Hrubá hmotnost vs B/L F202615259</t>
         </is>
       </c>
-      <c r="E23" s="17">
-        <f>F20</f>
+      <c r="F23" s="17">
+        <f>G20</f>
         <v>11430.0</v>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="G23" s="18" t="n">
         <v>11430</v>
       </c>
-      <c r="G23" s="19" t="str">
-        <f>IF(ROUND(E23-F23,2)=0,"OK","ROZDÍL / DIFF")</f>
+      <c r="H23" s="19" t="str">
+        <f>IF(ROUND(F23-G23,2)=0,"OK","ROZDÍL / DIFF")</f>
         <v>OK</v>
       </c>
     </row>
@@ -1105,15 +1135,15 @@
           <t>Čistá hmotnost vs balicí listy PL-504 + PL-902</t>
         </is>
       </c>
-      <c r="E24" s="17">
-        <f>E20</f>
+      <c r="F24" s="17">
+        <f>F20</f>
         <v>9643.0</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="G24" s="18" t="n">
         <v>9643</v>
       </c>
-      <c r="G24" s="19" t="str">
-        <f>IF(ROUND(E24-F24,2)=0,"OK","ROZDÍL / DIFF")</f>
+      <c r="H24" s="19" t="str">
+        <f>IF(ROUND(F24-G24,2)=0,"OK","ROZDÍL / DIFF")</f>
         <v>OK</v>
       </c>
     </row>
@@ -1123,15 +1153,15 @@
           <t>Celní hodnota vs faktury CI-26051504 + CI-26051902</t>
         </is>
       </c>
-      <c r="E25" s="17">
-        <f>I20</f>
+      <c r="F25" s="17">
+        <f>J20</f>
         <v>67063.32</v>
       </c>
-      <c r="F25" s="18" t="n">
+      <c r="G25" s="18" t="n">
         <v>67063.32000000001</v>
       </c>
-      <c r="G25" s="19" t="str">
-        <f>IF(ROUND(E25-F25,2)=0,"OK","ROZDÍL / DIFF")</f>
+      <c r="H25" s="19" t="str">
+        <f>IF(ROUND(F25-G25,2)=0,"OK","ROZDÍL / DIFF")</f>
         <v>OK</v>
       </c>
     </row>
@@ -1144,20 +1174,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="B8:K8"/>
-    <mergeCell ref="B4:K4"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B13:K13"/>
-    <mergeCell ref="B12:K12"/>
-    <mergeCell ref="B7:K7"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="B6:K6"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="B10:K10"/>
-    <mergeCell ref="B11:K11"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B12:L12"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="B6:L6"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="B7:L7"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="B8:L8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verify grouping against supplier's revised invoices with HS codes
Grandview reissued both invoices with the HS CODE column populated. Compared
line by line: 97 of 98 lines carry a code and all 97 agree with this summary -
8547 20 00 on 32 lines, 3917 40 00 on 12, 8547 90 00 on 53. Amounts and
quantities are unchanged, so no figures move.

The one line without a supplier code is line 78, the type wheel - now absent
from the packing list, the forwarder's e-mail and the supplier's own code list.
Three independent omissions support treating it as tooling that stays in China,
in which case the 120.00 USD is an assist under UCC Art. 71(1)(b)(ii) rather
than a separate declarable item.

Origin, Incoterm and the missing preferential statement are unchanged on the
revised invoices, so those flags stay open.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjrBV2HCzRFVHdsJfaktnd
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MOREK_CZ_CZ26008741.xlsx
+++ b/output/HS_Code_Summary_MOREK_CZ_CZ26008741.xlsx
@@ -10010,24 +10010,24 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="39" t="inlineStr">
-        <is>
-          <t>3. HS KÓDY NA FAKTURÁCH — prázdné</t>
-        </is>
-      </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>ZJIŠTĚNO</t>
-        </is>
-      </c>
-      <c r="C6" s="41" t="inlineStr">
-        <is>
-          <t>Obě faktury mají sloupec "HS CODE", ale je ve VŠECH řádcích prázdný — dodavatel jej nevyplnil. Klasifikaci jsem proto provedl sám (viz bod 4). Doporučuji vyžádat od dodavatele doplnění.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>3. HS KÓDY NA FAKTURÁCH — doplněny</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>OVĚŘENO</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Původní faktury měly sloupec "HS CODE" prázdný ve všech řádcích. Dodavatel následně vydal REVIDOVANÉ faktury (CI26051504_HScodes, CI26051902_HScodes) s HS kódem u každé položky. Provedl jsem porovnání položku po položce: 97 z 98 řádků má kód vyplněný a VŠECH 97 se shoduje s tímto souhrnem — 8547 20 00 u 32 řádků (HW, MW-A, MW-U), 3917 40 00 u 12 řádků (sady MSTS), 8547 90 00 u 53 řádků (tenkostěnná). Zařazení podle skupin tedy sedí na 100 %. Částky ani množství se na revidovaných fakturách nezměnily (celkem 67 063,32 USD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
       <c r="A7" s="42" t="inlineStr">
         <is>
           <t>4. POUŽITÉ HS KÓDY — dle speditéra</t>
@@ -10040,7 +10040,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Souhrn je sestaven podle tří kódů z e-mailu Maurice Ward (L. Jirkovský, ref. OR / MOREK / ASV20260522011 / CZ26008741): 8547 20 00 = smršťovací trubice silnostěnná a středněstěnná (skupiny HW, MW-A, MW-U); 3917 40 00 = spojovací set (skupina KIT — sady MSTS); 8547 90 00 = smršťovací bužírka tenkostěnná (skupina TW). České popisy jsou převzaty doslovně z jeho e-mailu.</t>
+          <t>Souhrn je sestaven podle tří kódů z e-mailu Maurice Ward (L. Jirkovský, ref. OR / MOREK / ASV20260522011 / CZ26008741): 8547 20 00 = smršťovací trubice silnostěnná a středněstěnná (skupiny HW, MW-A, MW-U); 3917 40 00 = spojovací set (skupina KIT — sady MSTS); 8547 90 00 = smršťovací bužírka tenkostěnná (skupina TW). České popisy jsou převzaty doslovně z jeho e-mailu. POTVRZENO: dodavatel mezitím doplnil HS kódy přímo do faktur a u všech 97 zbožových řádků uvádí tytéž tři kódy ve stejném rozdělení (viz bod 3) — speditér a dodavatel se shodují.</t>
         </is>
       </c>
     </row>
@@ -10112,7 +10112,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="78" customHeight="1">
+    <row r="12" ht="130" customHeight="1">
       <c r="A12" s="44" t="inlineStr">
         <is>
           <t>6. TYPE WHEEL — 3 ks, chybí všude</t>
@@ -10125,7 +10125,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Faktura CI-26051504, řádek 78: "type wheel", 3 ks, 40,00 USD/ks = 120,00 USD. Tato položka NENÍ v balicím listu PL-504 (fakturováno 112 548 ks vs. baleno 112 545 ks — rozdíl přesně 3 ks) a NENÍ ani v e-mailu speditéra, který uvádí jen tři kódy pro trubice, bužírky a sety. Nemá tedy žádnou hmotnost a čtvrtý kód pro ni nikdo nestanovil. Podle povahy buď 8442 50 00 (tiskařské typy/štočky), nebo 8443 99 (části tiskáren). Prosím o upřesnění, co to je, zda je fyzicky v zásilce a pod jakým kódem se má deklarovat.</t>
+          <t>Faktura CI-26051504, řádek 78: "type wheel", 3 ks, 40,00 USD/ks = 120,00 USD. Tato položka NENÍ v balicím listu PL-504 (fakturováno 112 548 ks vs. baleno 112 545 ks — rozdíl přesně 3 ks), NENÍ v e-mailu speditéra, a na REVIDOVANÉ faktuře s HS kódy ji dodavatel jako JEDINOU ZE VŠECH 98 řádků nechal BEZ KÓDU. Tři nezávislé zdroje ji tedy vynechávají — to podporuje výklad, že nejde o zasílané zboží, ale o nářadí (tiskové kolečko na potisk trubic), které zůstává u dodavatele. V takovém případě se nedeklaruje samostatně a 120,00 USD se podle čl. 71 odst. 1 písm. b) bodu ii) celního kodexu Unie připočte k celní hodnotě potištěného zboží. Pokud se přesto fyzicky veze, připadá v úvahu 8442 50 00 (tiskařské pomůcky), případně 8443 99 (části tiskových strojů). Podle povahy buď 8442 50 00 (tiskařské typy/štočky), nebo 8443 99 (části tiskáren). Prosím o upřesnění, co to je, zda je fyzicky v zásilce a pod jakým kódem se má deklarovat.</t>
         </is>
       </c>
     </row>

</xml_diff>